<commit_message>
Docs, deck and workbook: current state — reputation per skill, review proof, VPS hosting and backups, 857 tests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -49,12 +49,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="009A6A00"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="009A6A00"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -102,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -128,16 +128,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -634,11 +631,11 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Deploy left (you)</t>
+          <t>Done (live on VPS)</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>24</v>
@@ -698,14 +695,14 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Deploy left (you)</t>
+          <t>Done (live on Vercel)</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G6" s="5">
         <f>IF(F6=0,0,E6/F6)</f>
@@ -730,14 +727,14 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Video left (you)</t>
+          <t>Backup video left (you)</t>
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G7" s="5">
         <f>IF(F7=0,0,E7/F7)</f>
@@ -760,13 +757,13 @@
           <t>Oct 12-13</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>In progress (video done)</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>8</v>
@@ -777,23 +774,23 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="10">
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="9">
         <f>SUM(E2:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="9">
         <f>SUM(F2:F8)</f>
         <v/>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="11">
         <f>IF(F9=0,0,E9/F9)</f>
         <v/>
       </c>
@@ -958,14 +955,14 @@
           <t>Sep 22</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Deferred to M5 by the owner's earlier call.</t>
+          <t>Cleared Oct 7: backend on a Vultr VPS behind Caddy (https://api.64-177-41-175.sslip.io), site on Vercel (https://agentx-interface-iota.vercel.app); 16/16 deployment checks, three runs from the site settled. Railway not used (trial expired).</t>
         </is>
       </c>
     </row>
@@ -995,7 +992,7 @@
           <t>Sep 28</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1032,14 +1029,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Must be public by Oct 13; the submission requires a code link.</t>
+          <t>Public since Oct 6: agentx-contracts, agentx-backend, agentx-interface, agentx-docs (branch master).</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1337,7 +1334,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
@@ -1357,7 +1354,7 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
@@ -1377,7 +1374,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
@@ -1397,7 +1394,7 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
@@ -1597,7 +1594,7 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
@@ -1637,7 +1634,7 @@
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
@@ -1717,7 +1714,7 @@
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
@@ -1988,100 +1985,100 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>agentx-interface</t>
+          <t>agentx-backend</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>lib/api + subscribe</t>
+          <t>api/skills</t>
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>formatUnits past 2^53; SSE kinds, bad frames; only a terminal event ends a run; reconnect + replay reset; 5xx/503 read as sentences</t>
+          <t>Per-skill reputation: a proven specialist ranks first for its skill even below a stronger generalist overall; counts what the indexer counts; every skill on the profile</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>agentx-interface</t>
+          <t>agentx-backend</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>lib/search</t>
+          <t>db/reputation</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Docs search: typos, stems, synonyms, identifiers, AND, ranking, hostile input, sections from HTML</t>
+          <t>One shared score formula, identical to the indexer's for every history; no history scores 50; worker-fault reasons</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>agentx-interface</t>
+          <t>agentx-backend</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>lib/links</t>
+          <t>agent-core/model-failure</t>
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>Explorer links: https + known host only; uuid and agent id parsing</t>
+          <t>A used-up quota, a 429, overload and timeouts, a rejected key each named as such</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>agentx-interface</t>
+          <t>agentx-backend</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>components</t>
+          <t>agent-core/recordings</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>RunTrace (hostile links, money, live region), NetworkBadge (never assumes testnet)</t>
+          <t>Every committed model recording is still reachable from the current prompts, so the cached demo cannot silently break</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>agentx-interface</t>
+          <t>agentx-backend</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>lib/wallet</t>
+          <t>agent-core/judge</t>
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>Addresses and RPC validated before the wallet is asked; chain added on 4902</t>
+          <t>The judge rates a step against its own subtask, not the whole goal</t>
         </is>
       </c>
     </row>
@@ -2093,15 +2090,15 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>lib/agent-card</t>
+          <t>lib/api + subscribe</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>ERC-8004 registration-v1 card and its data: URI, non-ASCII safe</t>
+          <t>formatUnits past 2^53; SSE kinds, bad frames; only a terminal event ends a run; reconnect + replay reset; 5xx/503 read as sentences</t>
         </is>
       </c>
     </row>
@@ -2113,26 +2110,166 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
+          <t>lib/search</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Docs search: typos, stems, synonyms, identifiers, AND, ranking, hostile input, sections from HTML</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>lib/links</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Explorer links: https + known host only; uuid and agent id parsing</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>components</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>RunTrace (hostile links, money, live region), NetworkBadge (never assumes testnet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>lib/wallet</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Addresses and RPC validated before the wallet is asked; chain added on 4902</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>lib/agent-card</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>ERC-8004 registration-v1 card and its data: URI, non-ASCII safe</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
           <t>lib/format</t>
         </is>
       </c>
-      <c r="C53" s="6" t="n">
+      <c r="C58" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D53" s="8" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>Relative time and durations, refusing nonsense input</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="14" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>lib/review</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>The on-chain review under a settled step: links the settlement transaction, says so when the registry refused, claims nothing before indexing or for a refund</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>agentx-interface</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>components/StepList</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Every step status as a label with its reason, never a code</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="13" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C54" s="10">
-        <f>SUM(C2:C53)</f>
+      <c r="C61" s="9">
+        <f>SUM(C2:C60)</f>
         <v/>
       </c>
     </row>
@@ -3487,7 +3624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3527,12 +3664,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Deploy</t>
+          <t>Contracts</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Railway (api, signer, indexer) + Vercel</t>
+          <t>Verify source on the explorer</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -3547,7 +3684,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Follow docs/13-deploy.md; then node scripts/check-deployment.mjs &lt;api&gt; &lt;site&gt;.</t>
+          <t>Needs EXPLORER_API_KEY; the config defect is fixed.</t>
         </is>
       </c>
     </row>
@@ -3559,7 +3696,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>2-3 minute video</t>
+          <t>Fill the portal and submit</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -3569,24 +3706,24 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Record the cached replay (v2 Ollama recording of Sep 30; 162 s with AGENT_REPLAY_MAX_MS=2000) and the interface. Claude cannot record video.</t>
+          <t>Field-by-field text in docs/18-portal-entry.md; the judges' orchestrator key goes in the private field only.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Contracts</t>
+          <t>Hosting</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Verify source on the explorer</t>
+          <t>Destroy the VPS after judging</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -3596,24 +3733,24 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Needs EXPLORER_API_KEY; the config defect is fixed.</t>
+          <t>It bills monthly once the credit ends. Daily database backups run on it (03:00 UTC, 7 kept).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Submit</t>
+          <t>Testnet</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Make the three repos public</t>
+          <t>Testnet MON for hosted runs</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -3623,64 +3760,37 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Required by Oct 13. Full-history scan for every real secret: clean (Sep 30).</t>
+          <t>A hosted run measured 0.21 MON; a local demo run ~0.5 MON. See PROGRESS for current balances; seed-hosted.mjs --top-up refills the hosted agents.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Testnet</t>
+          <t>Post-hack</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Testnet MON for the video run</t>
+          <t>ERC-8183 conformance: new kernel + AGENTX evaluator + hook</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>User</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P4</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>A demo run costs ~0.5 MON. See PROGRESS for current balances; 6 MON each moved from AGENT_A/B for v2, as allowed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Post-hack</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>ERC-8183 conformance: new kernel + AGENTX evaluator + hook</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Mapping written: docs/12. Needs a redeploy, so after the deadline.</t>
         </is>
@@ -3697,7 +3807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3748,7 +3858,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3803,10 +3913,58 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>Live site</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>https://agentx-interface-iota.vercel.app (Vercel, deploys from master)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Live API</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>https://api.64-177-41-175.sslip.io (Vultr VPS behind Caddy; daily database backup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>857 unit/integration (184 contracts, 586 backend, 87 interface) + 72 browser tests on 5 engines (360 runs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Repos</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>agentx-contracts, agentx-backend, agentx-interface, agentx-docs — public, branch master</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
           <t>Formulas</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Totals and percentages are formulas so the sheet recalculates when a count changes. They were NOT recalculated when written — that needs LibreOffice, which the build machine lacks — so Excel computes them on first open.</t>
         </is>

</xml_diff>

<commit_message>
Figures: 859 tests (588 backend) after the placeholder fix; Session 34 live checks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agentx-status.xlsx
+++ b/docs/agentx-status.xlsx
@@ -1334,7 +1334,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
@@ -3942,7 +3942,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>857 unit/integration (184 contracts, 586 backend, 87 interface) + 72 browser tests on 5 engines (360 runs)</t>
+          <t>859 unit/integration (184 contracts, 588 backend, 87 interface) + 72 browser tests on 5 engines (360 runs)</t>
         </is>
       </c>
     </row>

</xml_diff>